<commit_message>
Reword the consulting offer in Thomas's own voice
Applied identically in all three places the offer appears — the results page,
the completion email, and the Strategic Recommendations tab of the XLSX — and
rebuilt the frozen sample workbook so the downloadable sample matches.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/sample/kelvara-systems-grant-analysis.xlsx
+++ b/frontend/sample/kelvara-systems-grant-analysis.xlsx
@@ -1292,7 +1292,7 @@
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>Get help with these applications</t>
+          <t>Want help winning a grant?</t>
         </is>
       </c>
       <c r="B15" t="inlineStr"/>
@@ -1305,7 +1305,7 @@
       </c>
       <c r="B16" s="2" t="inlineStr">
         <is>
-          <t>Built by Thomas Murray, a consultant who helps climate and deeptech startups win grant funding. This shortlist is the same landscape scan I run at the start of a client engagement — if you want help turning any of these into a submitted application, get in touch.</t>
+          <t>I'm Thomas Murray. I help climate and deep tech startups win grant funding and achieve profitability. This tool is a productised version of an opportunity assessment I've done for several startups. If you want help turning a grant opportunity into a complete application, contact me.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
XLSX includes the watchlist, back-to-site header link, server-side auto-continue
The XLSX download only ever contained the scored shortlist, hiding the
strategic watchlist items that show on the results page — the "Grant
Opportunities" tab now includes both. Since the app is reached via a link
from thomasmurray.earth, the header now links back to it, with the
"Climate & deeptech funding intelligence" eyebrow moved down to sit above
the hero heading instead. The profile-review auto-continue timer moved
from the browser to the server, so grant discovery starts even if the
user closes the tab.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/sample/kelvara-systems-grant-analysis.xlsx
+++ b/frontend/sample/kelvara-systems-grant-analysis.xlsx
@@ -463,7 +463,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:X5"/>
+  <dimension ref="A1:X26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20.63" customWidth="1" min="1" max="1"/>
@@ -1062,8 +1062,2564 @@
         </is>
       </c>
     </row>
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem Long Duration Electricity Storage (LDES) Cap and Floor Regime — Window 2</t>
+        </is>
+      </c>
+      <c r="B6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C6" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem's LDES cap and floor regime is designed to de-risk long-duration energy storage projects in the UK grid — directly relevant to Kelvara's grid-scale thermal battery providing 8+ hour storage. Window 1 advanced 16 projects in June 2026; Window 2 is expected. This is the primary UK policy instrument for LDES commercialisation.</t>
+        </is>
+      </c>
+      <c r="D6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Concessional | Revenue support mechanism — project-specific; no fixed grant amount</t>
+        </is>
+      </c>
+      <c r="J6" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K6" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ofgem.gov.uk/decision/long-duration-electricity-storage-cap-and-floor-application-window-1</t>
+        </is>
+      </c>
+      <c r="L6" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem</t>
+        </is>
+      </c>
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q6" s="2" t="inlineStr">
+        <is>
+          <t>Completion of the 5 MWh commercial pilot and identification of a UK grid-connected deployment site would make Kelvara eligible to apply for Window 2 as a project entity seeking revenue support for a grid-scale LDES deployment.</t>
+        </is>
+      </c>
+      <c r="R6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S6" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T6" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U6" s="2" t="inlineStr">
+        <is>
+          <t>known future window</t>
+        </is>
+      </c>
+      <c r="V6" s="2" t="inlineStr">
+        <is>
+          <t>Window 2 application process not yet confirmed open, and the revenue support mechanism requires a grid-connected project at a scale and maturity likely beyond Kelvara's current 500 kWh demonstration — the application route is unclear for a seed-stage company.</t>
+        </is>
+      </c>
+      <c r="W6" s="2" t="inlineStr">
+        <is>
+          <t>Unclear Application Route</t>
+        </is>
+      </c>
+      <c r="X6" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>ARENA / AMGC Industrial Electrification Fund</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>The fund explicitly targets electrification of industrial processes reliant on fossil fuels for SME manufacturers — a direct thematic match for Kelvara's thermal battery enabling process heat electrification. Opens July 2026, assessed on a continuous basis until December 2027.</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I7" s="2" t="inlineStr">
+        <is>
+          <t>Grant | $10M total fund; individual grant amounts unknown</t>
+        </is>
+      </c>
+      <c r="J7" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K7" s="4" t="inlineStr">
+        <is>
+          <t>https://arena.gov.au/funding/</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Australian Renewable Energy Agency (ARENA) / Advanced Manufacturing Growth Centre (AMGC)</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q7" s="2" t="inlineStr">
+        <is>
+          <t>Establishing an Australian entity or partnering with an Australian industrial manufacturer as co-applicant would make this fund accessible — worth pursuing if Kelvara's Australia expansion progresses in 2026-2027.</t>
+        </is>
+      </c>
+      <c r="R7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S7" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T7" s="2" t="inlineStr">
+        <is>
+          <t>Australia</t>
+        </is>
+      </c>
+      <c r="U7" s="2" t="inlineStr">
+        <is>
+          <t>known future window</t>
+        </is>
+      </c>
+      <c r="V7" s="2" t="inlineStr">
+        <is>
+          <t>Kelvara lists Australia as only an exploratory geography with no confirmed operational presence or Australian-registered entity — the fund requires Australian SME manufacturers, creating a geography and entity eligibility barrier.</t>
+        </is>
+      </c>
+      <c r="W7" s="2" t="inlineStr">
+        <is>
+          <t>Direct Startup Application</t>
+        </is>
+      </c>
+      <c r="X7" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem Strategic Innovation Fund (SIF) — Discovery C6</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>SIF funds energy network innovation including grid flexibility and storage; Kelvara's thermal battery provides long-duration grid flexibility by absorbing surplus renewables, aligning with SIF's network innovation objectives.</t>
+        </is>
+      </c>
+      <c r="D8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I8" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J8" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K8" s="4" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2484/overview/770c0946-2e24-4566-bab1-2bf1c1dd2b38</t>
+        </is>
+      </c>
+      <c r="L8" s="2" t="inlineStr">
+        <is>
+          <t>Ofgem / Innovate UK</t>
+        </is>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q8" s="2" t="inlineStr">
+        <is>
+          <t>Identify a licensed or regulated organisation (network operator, NHS trust, housing association, or local authority) willing to act as lead applicant, with the startup named as the technology partner.</t>
+        </is>
+      </c>
+      <c r="R8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S8" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T8" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U8" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V8" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but not deep-researched. It likely requires a licensed or regulated entity (e.g. network operator, NHS trust, housing association, or local authority) as lead applicant. The startup may be able to participate as a named technology partner. Verify current eligibility and identify a suitable lead organisation.</t>
+        </is>
+      </c>
+      <c r="W8" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X8" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK Knowledge Transfer Partnership (KTP) — 2026-2027 Round 3 (anticipated)</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>KTP supports UK SMEs to embed academic expertise into innovation projects; Kelvara as a university spinout could use KTP to accelerate R&amp;D on PCM thermal storage with a UK university partner.</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I9" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J9" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K9" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ukri.org/councils/innovate-uk/guidance-for-applicants/guidance-for-specific-funds/knowledge-transfer-partnership-guidance/dates-and-deadlines-for-ktp-applicants/</t>
+        </is>
+      </c>
+      <c r="L9" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK / UKRI</t>
+        </is>
+      </c>
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q9" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S9" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T9" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U9" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V9" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W9" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X9" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="2" t="inlineStr">
+        <is>
+          <t>MBIE Strategic Science Investment Fund (SSIF) — Advanced Energy Technology Platform</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C10" s="2" t="inlineStr">
+        <is>
+          <t>SSIF Advanced Energy Technology Platform funds NZ-based advanced energy technology R&amp;D; Kelvara's aluminium-alloy PCM thermal battery is a novel advanced energy technology with NZ HQ.</t>
+        </is>
+      </c>
+      <c r="D10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I10" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J10" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K10" s="4" t="inlineStr">
+        <is>
+          <t>https://www.mbie.govt.nz/science-and-technology/science-and-innovation/funding-information-and-opportunities/investment-funds/strategic-science-investment-fund</t>
+        </is>
+      </c>
+      <c r="L10" s="2" t="inlineStr">
+        <is>
+          <t>Ministry of Business, Innovation and Employment (MBIE), New Zealand</t>
+        </is>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q10" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S10" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T10" s="2" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="U10" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V10" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W10" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X10" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="2" t="inlineStr">
+        <is>
+          <t>Callaghan Innovation — R&amp;D Project Grant (New Zealand)</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>Callaghan Innovation funds NZ-based SME R&amp;D projects; Kelvara's seed-stage thermal battery development with NZ HQ is a strong fit for project grant support.</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I11" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J11" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K11" s="4" t="inlineStr">
+        <is>
+          <t>https://www.callaghaninnovation.govt.nz/</t>
+        </is>
+      </c>
+      <c r="L11" s="2" t="inlineStr">
+        <is>
+          <t>Callaghan Innovation, New Zealand</t>
+        </is>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q11" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S11" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T11" s="2" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="U11" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V11" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W11" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X11" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>EIT InnoEnergy — Call for Proposals (Energy Storage / Industrial Decarbonisation)</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C12" s="2" t="inlineStr">
+        <is>
+          <t>EIT InnoEnergy explicitly funds energy storage, renewable energy, and energy efficiency innovations for industrial applications — core to Kelvara's thermal battery product.</t>
+        </is>
+      </c>
+      <c r="D12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Blended | unknown</t>
+        </is>
+      </c>
+      <c r="J12" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K12" s="4" t="inlineStr">
+        <is>
+          <t>https://innoenergy.com/</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>EIT InnoEnergy</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q12" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S12" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T12" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States and associated countries</t>
+        </is>
+      </c>
+      <c r="U12" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V12" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W12" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X12" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="inlineStr">
+        <is>
+          <t>UK Flexibility Innovation Programme — DESNZ</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>Programme supports innovative solutions for large-scale electricity system flexibility — directly relevant to Kelvara's thermal battery absorbing surplus renewables and providing grid flexibility.</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J13" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K13" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/publications/flexibility-innovation</t>
+        </is>
+      </c>
+      <c r="L13" s="2" t="inlineStr">
+        <is>
+          <t>Department for Energy Security and Net Zero (DESNZ)</t>
+        </is>
+      </c>
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q13" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S13" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T13" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U13" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V13" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W13" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X13" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Government — Industrial Energy Efficiency and Decarbonisation Fund</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C14" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Government fund supports industrial sites investing in energy efficiency and decarbonisation — directly aligned with Kelvara's thermal battery for industrial process heat replacement.</t>
+        </is>
+      </c>
+      <c r="D14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I14" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K14" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gov.scot/collections/scottish-industrial-energy-transformation-fund-sietf/</t>
+        </is>
+      </c>
+      <c r="L14" s="2" t="inlineStr">
+        <is>
+          <t>Scottish Government / Scottish Enterprise</t>
+        </is>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q14" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S14" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T14" s="2" t="inlineStr">
+        <is>
+          <t>Scotland, United Kingdom</t>
+        </is>
+      </c>
+      <c r="U14" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V14" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W14" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X14" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="2" t="inlineStr">
+        <is>
+          <t>UKRI Net Zero Industrial Decarbonisation Challenge — specific competition (2026-2027)</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>UKRI's industrial decarbonisation challenge funds target exactly the sectors Kelvara serves (food, chemicals, paper) and the technology approach (electrification of process heat).</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J15" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K15" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ukri.org/councils/innovate-uk/</t>
+        </is>
+      </c>
+      <c r="L15" s="2" t="inlineStr">
+        <is>
+          <t>UKRI / Innovate UK</t>
+        </is>
+      </c>
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q15" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S15" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T15" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U15" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V15" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W15" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X15" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK — Next Wave: Breakthrough Wave 1</t>
+        </is>
+      </c>
+      <c r="B16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C16" s="2" t="inlineStr">
+        <is>
+          <t>Programme supports UK SMEs developing breakthrough technologies at the intersection of deep tech and UK Industrial Strategy priorities, which includes net zero and energy — relevant to Kelvara's deep tech thermal battery.</t>
+        </is>
+      </c>
+      <c r="D16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I16" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K16" s="4" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/2517/overview/6ff2066d-4639-44e6-bb4f-ce7099222739</t>
+        </is>
+      </c>
+      <c r="L16" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK / UKRI</t>
+        </is>
+      </c>
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q16" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S16" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T16" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U16" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V16" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W16" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X16" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>EU Innovation Fund — Large-Scale Projects Call (next round, 2026-2027)</t>
+        </is>
+      </c>
+      <c r="B17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>Innovation Fund large-scale calls fund highly innovative low-carbon technologies including energy storage and industrial decarbonisation — strong alignment with Kelvara's grid-scale thermal battery.</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I17" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J17" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K17" s="4" t="inlineStr">
+        <is>
+          <t>https://cinea.ec.europa.eu/programmes/innovation-fund_en</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>European Commission (Innovation Fund / CINEA)</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q17" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S17" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T17" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States and EEA/associated countries</t>
+        </is>
+      </c>
+      <c r="U17" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V17" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W17" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X17" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK — Sustainable Innovation Fund / Net Zero Transition Fund (2026-2027 round)</t>
+        </is>
+      </c>
+      <c r="B18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C18" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK net zero transition competitions fund UK SMEs developing clean energy and decarbonisation technologies — directly relevant to Kelvara's thermal battery for industrial emissions reduction.</t>
+        </is>
+      </c>
+      <c r="D18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I18" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K18" s="4" t="inlineStr">
+        <is>
+          <t>https://apply-for-innovation-funding.service.gov.uk/competition/search</t>
+        </is>
+      </c>
+      <c r="L18" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK / UKRI</t>
+        </is>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q18" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S18" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T18" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U18" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V18" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W18" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X18" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Horizon Europe — Processes4Planet Partnership (industrial process decarbonisation)</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>Processes4Planet targets optimisation of energy and materials use in industrial processes including recycling and upcycling — partial alignment with Kelvara's circular economy use of recycled aluminium and industrial process heat.</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I19" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J19" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K19" s="4" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/opportunities/calls-for-proposals?callIdentifier=HORIZON-CID-2027-01</t>
+        </is>
+      </c>
+      <c r="L19" s="2" t="inlineStr">
+        <is>
+          <t>European Commission / Horizon Europe</t>
+        </is>
+      </c>
+      <c r="M19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q19" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S19" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T19" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States and associated countries</t>
+        </is>
+      </c>
+      <c r="U19" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V19" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W19" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X19" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t>UK Research Fund for Coal and Steel (RFCS) — complementary call via Horizon Europe</t>
+        </is>
+      </c>
+      <c r="B20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C20" s="2" t="inlineStr">
+        <is>
+          <t>RFCS funds decarbonisation of energy-intensive industries including steel and chemicals — sectors where Kelvara's thermal battery could displace fossil-fuel process heat, though primary focus is coal/steel sector.</t>
+        </is>
+      </c>
+      <c r="D20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I20" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K20" s="4" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/programmes/rfcs</t>
+        </is>
+      </c>
+      <c r="L20" s="2" t="inlineStr">
+        <is>
+          <t>European Commission</t>
+        </is>
+      </c>
+      <c r="M20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q20" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S20" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T20" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States</t>
+        </is>
+      </c>
+      <c r="U20" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V20" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W20" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X20" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK — Industrial Decarbonisation Challenge (IDC) follow-on competitions</t>
+        </is>
+      </c>
+      <c r="B21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>IDC aims to establish net-zero carbon industrial clusters in the UK; Kelvara's thermal battery enabling industrial process heat decarbonisation is a core enabling technology for this mission.</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I21" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J21" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K21" s="4" t="inlineStr">
+        <is>
+          <t>https://www.ukri.org/what-we-do/browse-our-areas-of-investment-and-support/industrial-decarbonisation/</t>
+        </is>
+      </c>
+      <c r="L21" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK / UKRI</t>
+        </is>
+      </c>
+      <c r="M21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q21" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S21" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T21" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U21" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V21" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W21" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X21" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>New Zealand Green Investment Finance (NZGIF) — Concessional Finance for Industrial Decarbonisation</t>
+        </is>
+      </c>
+      <c r="B22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C22" s="2" t="inlineStr">
+        <is>
+          <t>NZGIF provides concessional finance to accelerate NZ's transition to a low-emissions economy; Kelvara's industrial thermal battery for NZ industrial decarbonisation is within its mandate.</t>
+        </is>
+      </c>
+      <c r="D22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I22" s="2" t="inlineStr">
+        <is>
+          <t>Concessional | unknown</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K22" s="4" t="inlineStr">
+        <is>
+          <t>https://nzgif.co.nz/</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>New Zealand Green Investment Finance (NZGIF)</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q22" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S22" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T22" s="2" t="inlineStr">
+        <is>
+          <t>New Zealand</t>
+        </is>
+      </c>
+      <c r="U22" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V22" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W22" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X22" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Breakthrough Energy Fellows / Breakthrough Energy Ventures — Catalyst Programme</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>Breakthrough Energy Catalyst funds first-of-kind clean energy projects including long-duration storage and industrial decarbonisation — directly aligned with Kelvara's thermal battery technology.</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I23" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J23" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K23" s="4" t="inlineStr">
+        <is>
+          <t>https://breakthroughenergy.org/our-work/catalyst/</t>
+        </is>
+      </c>
+      <c r="L23" s="2" t="inlineStr">
+        <is>
+          <t>Breakthrough Energy</t>
+        </is>
+      </c>
+      <c r="M23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q23" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S23" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T23" s="2" t="inlineStr">
+        <is>
+          <t>Global</t>
+        </is>
+      </c>
+      <c r="U23" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V23" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W23" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X23" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="2" t="inlineStr">
+        <is>
+          <t>Horizon Europe — Battery Partnership (Batteries2030+ / BATT4EU) — Energy Storage Innovation</t>
+        </is>
+      </c>
+      <c r="B24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C24" s="2" t="inlineStr">
+        <is>
+          <t>Battery partnership calls include energy storage innovation beyond lithium-ion; Kelvara's aluminium-alloy PCM thermal battery as a novel grid-scale storage medium has partial fit, though primary focus is electrochemical batteries.</t>
+        </is>
+      </c>
+      <c r="D24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="E24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I24" s="2" t="inlineStr">
+        <is>
+          <t>Grant | unknown</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K24" s="4" t="inlineStr">
+        <is>
+          <t>https://ec.europa.eu/info/funding-tenders/opportunities/portal/screen/programmes/horizon</t>
+        </is>
+      </c>
+      <c r="L24" s="2" t="inlineStr">
+        <is>
+          <t>European Commission / Horizon Europe</t>
+        </is>
+      </c>
+      <c r="M24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q24" s="2" t="inlineStr">
+        <is>
+          <t>Review the programme's eligibility criteria and application process directly to determine whether the startup can apply.</t>
+        </is>
+      </c>
+      <c r="R24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S24" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T24" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States and associated countries</t>
+        </is>
+      </c>
+      <c r="U24" s="2" t="inlineStr">
+        <is>
+          <t>timing unknown</t>
+        </is>
+      </c>
+      <c r="V24" s="2" t="inlineStr">
+        <is>
+          <t>This programme was identified during discovery but was not selected for deep research. It showed partial thematic fit — verify eligibility and application process directly.</t>
+        </is>
+      </c>
+      <c r="W24" s="2" t="inlineStr">
+        <is>
+          <t>Direct applicant</t>
+        </is>
+      </c>
+      <c r="X24" s="2" t="inlineStr">
+        <is>
+          <t>Recurring</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="2" t="inlineStr">
+        <is>
+          <t>EIC Accelerator Open — Deep Tech for Climate Adaptation Challenge (2026)</t>
+        </is>
+      </c>
+      <c r="B25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>The named 'Deep Tech for Climate Adaptation' challenge is a direct match for Kelvara's climate hardware for industrial decarbonisation — a high-risk, deep-tech thermal battery at TRL 6 seeking commercialisation funding is precisely the EIC Accelerator's intended beneficiary.</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I25" s="2" t="inlineStr">
+        <is>
+          <t>Blended | Up to €2.5M grant + up to €15M equity (grant-only track available)</t>
+        </is>
+      </c>
+      <c r="J25" s="3" t="n">
+        <v>2500000</v>
+      </c>
+      <c r="K25" s="4" t="inlineStr">
+        <is>
+          <t>https://eic.ec.europa.eu/eic-funding-opportunities/eic-accelerator/eic-accelerator-challenges-2026/deep-tech-climate-adaptation_en</t>
+        </is>
+      </c>
+      <c r="L25" s="2" t="inlineStr">
+        <is>
+          <t>European Innovation Council (EIC)</t>
+        </is>
+      </c>
+      <c r="M25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q25" s="2" t="inlineStr">
+        <is>
+          <t>The next application round opening — monitor the programme page and prepare the application in advance.</t>
+        </is>
+      </c>
+      <c r="R25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S25" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T25" s="2" t="inlineStr">
+        <is>
+          <t>EU Member States and associated countries (UK associated)</t>
+        </is>
+      </c>
+      <c r="U25" s="2" t="inlineStr">
+        <is>
+          <t>open now</t>
+        </is>
+      </c>
+      <c r="V25" s="2" t="inlineStr">
+        <is>
+          <t>Well-established recurring programme with no application window currently open. The EIC Accelerator is a well-known, institutionalised recurring EU fund with confirmed 2026 Challenges rounds; the current_link points directly to the specific Deep Tech for Climate Adaptation challenge page, and no contradicting evidence suggests it has been cancelled.</t>
+        </is>
+      </c>
+      <c r="W25" s="2" t="inlineStr">
+        <is>
+          <t>Direct Startup Application</t>
+        </is>
+      </c>
+      <c r="X25" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK — Industrial Energy Transformation Fund (IETF) Phase 4</t>
+        </is>
+      </c>
+      <c r="B26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="C26" s="2" t="inlineStr">
+        <is>
+          <t>IETF's primary purpose is funding capital investment in industrial energy efficiency and heat decarbonisation — Kelvara's thermal battery for replacing fossil-fuel process heat is a textbook IETF project.</t>
+        </is>
+      </c>
+      <c r="D26" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="E26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="F26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="G26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="H26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I26" s="2" t="inlineStr">
+        <is>
+          <t>Grant | Up to £14.5M per project (feasibility: up to £80K; capital: up to £14.5M)</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="K26" s="4" t="inlineStr">
+        <is>
+          <t>https://www.gov.uk/government/collections/industrial-energy-transformation-fund</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Innovate UK / Department for Energy Security and Net Zero (DESNZ)</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="N26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="O26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="P26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="Q26" s="2" t="inlineStr">
+        <is>
+          <t>The next application round opening — monitor the programme page and prepare the application in advance.</t>
+        </is>
+      </c>
+      <c r="R26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="S26" s="2" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="T26" s="2" t="inlineStr">
+        <is>
+          <t>United Kingdom</t>
+        </is>
+      </c>
+      <c r="U26" s="2" t="inlineStr">
+        <is>
+          <t>open now</t>
+        </is>
+      </c>
+      <c r="V26" s="2" t="inlineStr">
+        <is>
+          <t>Well-established recurring programme with no application window currently open. The IETF is a well-established recurring UK government fund with multiple prior phases; search results returned no relevant evidence, but the programme's documented history of open rounds and the official GOV.UK collection page support a 'likely' status.</t>
+        </is>
+      </c>
+      <c r="W26" s="2" t="inlineStr">
+        <is>
+          <t>Direct Startup Application</t>
+        </is>
+      </c>
+      <c r="X26" s="2" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <conditionalFormatting sqref="B2:B5">
+  <conditionalFormatting sqref="B2:B26">
     <cfRule type="colorScale" priority="1">
       <colorScale>
         <cfvo type="min"/>
@@ -1073,7 +3629,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="D2:D5">
+  <conditionalFormatting sqref="D2:D26">
     <cfRule type="colorScale" priority="2">
       <colorScale>
         <cfvo type="min"/>
@@ -1083,7 +3639,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F2:F5">
+  <conditionalFormatting sqref="F2:F26">
     <cfRule type="colorScale" priority="3">
       <colorScale>
         <cfvo type="min"/>
@@ -1093,7 +3649,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="H2:H5">
+  <conditionalFormatting sqref="H2:H26">
     <cfRule type="colorScale" priority="4">
       <colorScale>
         <cfvo type="min"/>
@@ -1103,7 +3659,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J5">
+  <conditionalFormatting sqref="J2:J26">
     <cfRule type="colorScale" priority="5">
       <colorScale>
         <cfvo type="min"/>
@@ -1113,7 +3669,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N5">
+  <conditionalFormatting sqref="N2:N26">
     <cfRule type="expression" priority="6" dxfId="0">
       <formula>AND(ISNUMBER(N2),TRUNC(N2)&lt;TODAY())</formula>
     </cfRule>
@@ -1123,6 +3679,27 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K3" r:id="rId2"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K4" r:id="rId3"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K5" r:id="rId4"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K6" r:id="rId5"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K7" r:id="rId6"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K8" r:id="rId7"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K9" r:id="rId8"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K10" r:id="rId9"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K11" r:id="rId10"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K12" r:id="rId11"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K13" r:id="rId12"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K14" r:id="rId13"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K15" r:id="rId14"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K16" r:id="rId15"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K17" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K18" r:id="rId17"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K19" r:id="rId18"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K20" r:id="rId19"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K21" r:id="rId20"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K22" r:id="rId21"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K23" r:id="rId22"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K24" r:id="rId23"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K25" r:id="rId24"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="K26" r:id="rId25"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Give watchlist rows a real Priority Score in the XLSX
Watchlist grants never go through the full 3-axis scoring rubric, so
after the watchlist was folded into the XLSX, its rows showed "unknown"
for every score column. The discovery-stage thematic-fit rating computed
for every longlist candidate was being discarded rather than carried
through, so exporter.py had nothing to show. Backfill that rating onto
watchlist items (analyzer.py), and default Strategic Value / Ease of
Execution to 0 rather than "unknown" so the Priority Score formula
computes wherever a thematic fit rating exists at all.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/frontend/sample/kelvara-systems-grant-analysis.xlsx
+++ b/frontend/sample/kelvara-systems-grant-analysis.xlsx
@@ -1088,20 +1088,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F6" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H6" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H6" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I6" s="2" t="inlineStr">
         <is>
@@ -1210,20 +1206,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F7" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H7" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H7" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
@@ -1332,20 +1324,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H8" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H8" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
@@ -1454,20 +1442,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F9" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H9" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H9" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
@@ -1576,20 +1560,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F10" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H10" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H10" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
@@ -1698,20 +1678,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F11" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H11" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H11" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
@@ -1820,20 +1796,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F12" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H12" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H12" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I12" s="2" t="inlineStr">
         <is>
@@ -1942,20 +1914,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F13" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H13" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H13" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I13" s="2" t="inlineStr">
         <is>
@@ -2064,20 +2032,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F14" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H14" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H14" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
@@ -2186,20 +2150,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F15" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H15" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H15" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I15" s="2" t="inlineStr">
         <is>
@@ -2308,20 +2268,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H16" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H16" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
@@ -2430,20 +2386,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F17" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H17" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H17" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
@@ -2552,20 +2504,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F18" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F18" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H18" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H18" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
@@ -2674,20 +2622,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F19" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H19" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H19" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I19" s="2" t="inlineStr">
         <is>
@@ -2796,20 +2740,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F20" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F20" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H20" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H20" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I20" s="2" t="inlineStr">
         <is>
@@ -2918,20 +2858,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F21" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F21" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H21" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H21" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I21" s="2" t="inlineStr">
         <is>
@@ -3040,20 +2976,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F22" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F22" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H22" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H22" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I22" s="2" t="inlineStr">
         <is>
@@ -3162,20 +3094,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F23" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F23" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H23" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H23" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I23" s="2" t="inlineStr">
         <is>
@@ -3284,20 +3212,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F24" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F24" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H24" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H24" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I24" s="2" t="inlineStr">
         <is>
@@ -3386,10 +3310,9 @@
           <t>EIC Accelerator Open — Deep Tech for Climate Adaptation Challenge (2026)</t>
         </is>
       </c>
-      <c r="B25" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="B25" s="2">
+        <f>(2*D25)+F25+H25</f>
+        <v/>
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
@@ -3404,20 +3327,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F25" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F25" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H25" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H25" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I25" s="2" t="inlineStr">
         <is>
@@ -3504,10 +3423,9 @@
           <t>Innovate UK — Industrial Energy Transformation Fund (IETF) Phase 4</t>
         </is>
       </c>
-      <c r="B26" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="B26" s="2">
+        <f>(2*D26)+F26+H26</f>
+        <v/>
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
@@ -3522,20 +3440,16 @@
           <t>unknown</t>
         </is>
       </c>
-      <c r="F26" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="F26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
           <t>unknown</t>
         </is>
       </c>
-      <c r="H26" s="2" t="inlineStr">
-        <is>
-          <t>unknown</t>
-        </is>
+      <c r="H26" s="2" t="n">
+        <v>0</v>
       </c>
       <c r="I26" s="2" t="inlineStr">
         <is>

</xml_diff>